<commit_message>
2026-10-19: edits and additions
</commit_message>
<xml_diff>
--- a/RACI_Templates.xlsx
+++ b/RACI_Templates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waterfall RACI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agile RACI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Waterfall RACI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Agile RACI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -107,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -129,11 +129,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -182,6 +226,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,10 +618,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Copy this tab per project. Replace phase names/rows and roles as needed — keep one A per row.</t>
-        </is>
-      </c>
-    </row>
+          <t>Copy this tab per project. Replace phase names/rows and roles as needed - keep one A per row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -639,6 +686,15 @@
           <t>Initiation</t>
         </is>
       </c>
+      <c r="B5" s="18" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -666,26 +722,14 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I6" s="10" t="n"/>
       <c r="J6" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -705,7 +749,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -713,26 +757,10 @@
           <t>C</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
       <c r="I7" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -740,7 +768,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -780,21 +808,9 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H8" s="10" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -802,6 +818,15 @@
           <t>Requirements</t>
         </is>
       </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -809,11 +834,7 @@
           <t>Requirements gathering</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B10" s="10" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
           <t>A</t>
@@ -943,11 +964,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H12" s="10" t="n"/>
       <c r="I12" s="10" t="inlineStr">
         <is>
           <t>I</t>
@@ -965,6 +982,15 @@
           <t>Design</t>
         </is>
       </c>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -972,14 +998,10 @@
           <t>Solution/technical design</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B14" s="10" t="n"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -989,7 +1011,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1007,16 +1029,8 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I14" s="10" t="n"/>
+      <c r="J14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1059,16 +1073,8 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1076,21 +1082,13 @@
           <t>Security/architecture review</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B16" s="10" t="n"/>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n"/>
       <c r="E16" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1108,19 +1106,11 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>A/R</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1128,6 +1118,15 @@
           <t>Development</t>
         </is>
       </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1135,21 +1134,13 @@
           <t>Build/development</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B18" s="10" t="n"/>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n"/>
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1157,7 +1148,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1165,21 +1156,9 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1187,21 +1166,9 @@
           <t>Code review</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
       <c r="E19" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1209,7 +1176,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1222,16 +1189,8 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1239,29 +1198,13 @@
           <t>Unit testing</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -1269,21 +1212,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1291,6 +1222,15 @@
           <t>Testing</t>
         </is>
       </c>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="18" t="n"/>
+      <c r="J21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1298,14 +1238,10 @@
           <t>Test plan development</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B22" s="10" t="n"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -1325,7 +1261,7 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1333,16 +1269,8 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I22" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1350,14 +1278,10 @@
           <t>System integration testing</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B23" s="10" t="n"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -1377,7 +1301,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -1385,16 +1309,8 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I23" s="10" t="n"/>
+      <c r="J23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1417,11 +1333,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="E24" s="10" t="n"/>
       <c r="F24" s="10" t="inlineStr">
         <is>
           <t>I</t>
@@ -1432,11 +1344,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H24" s="10" t="n"/>
       <c r="I24" s="10" t="inlineStr">
         <is>
           <t>I</t>
@@ -1454,21 +1362,13 @@
           <t>Defect resolution</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B25" s="10" t="n"/>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="n"/>
       <c r="E25" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1476,7 +1376,7 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -1484,21 +1384,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="J25" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="10" t="n"/>
+      <c r="J25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1506,6 +1394,15 @@
           <t>Deployment</t>
         </is>
       </c>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="18" t="n"/>
+      <c r="I26" s="18" t="n"/>
+      <c r="J26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1624,14 +1521,10 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n"/>
       <c r="E29" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1639,7 +1532,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -1647,11 +1540,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H29" s="10" t="n"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1669,6 +1558,15 @@
           <t>Closure</t>
         </is>
       </c>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1716,11 +1614,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="J31" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="J31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -1758,22 +1652,15 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H32" s="10" t="n"/>
+      <c r="I32" s="10" t="n"/>
       <c r="J32" s="10" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
@@ -1789,7 +1676,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Responsible — does the work to complete the task</t>
+          <t>Responsible - does the work to complete the task</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1688,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Accountable — owns the outcome, signs off, single owner per row</t>
+          <t>Accountable - owns the outcome, signs off, single owner per row</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1700,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Consulted — two-way input sought before/during the work</t>
+          <t>Consulted - two-way input sought before/during the work</t>
         </is>
       </c>
     </row>
@@ -1825,10 +1712,11 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Informed — kept updated on progress or outcome, one-way</t>
-        </is>
-      </c>
-    </row>
+          <t>Informed - kept updated on progress or outcome, one-way</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
@@ -1839,7 +1727,7 @@
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>- If a role has no R/A/C/I on a row, leave the cell blank — do not mark every role on every row.</t>
+          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
         </is>
       </c>
     </row>
@@ -1903,10 +1791,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Copy this tab per team/program. Substitute Scrum roles for Kanban/SAFe as needed — keep one A per row.</t>
-        </is>
-      </c>
-    </row>
+          <t>Copy this tab per team/program. Substitute Scrum roles for Kanban/SAFe as needed - never more than one A per row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1966,6 +1855,14 @@
           <t>Program/Release Setup</t>
         </is>
       </c>
+      <c r="B5" s="18" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1975,7 +1872,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>R, A</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1988,11 +1885,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="E6" s="10" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -2003,14 +1896,10 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H6" s="10" t="n"/>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -2082,26 +1971,14 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="E8" s="10" t="n"/>
       <c r="F8" s="10" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="10" t="n"/>
       <c r="I8" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -2114,11 +1991,19 @@
           <t>Sprint Cadence</t>
         </is>
       </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Backlog refinement/grooming</t>
+          <t>Backlog refinement</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -2128,12 +2013,12 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2146,21 +2031,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2198,16 +2071,8 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2215,11 +2080,7 @@
           <t>Daily standup</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B12" s="10" t="n"/>
       <c r="C12" s="8" t="inlineStr">
         <is>
           <t>R</t>
@@ -2235,26 +2096,10 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2287,21 +2132,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="10" t="n"/>
+      <c r="I13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -2309,16 +2142,8 @@
           <t>Development</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
       <c r="D14" s="8" t="inlineStr">
         <is>
           <t>R</t>
@@ -2334,21 +2159,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2356,16 +2169,8 @@
           <t>Code review</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
       <c r="D15" s="8" t="inlineStr">
         <is>
           <t>R</t>
@@ -2381,21 +2186,13 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G15" s="10" t="n"/>
       <c r="H15" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2403,6 +2200,14 @@
           <t>Quality &amp; Review</t>
         </is>
       </c>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2415,11 +2220,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="C17" s="10" t="n"/>
       <c r="D17" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -2427,29 +2228,17 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>R, A</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
       <c r="H17" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="I17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2462,11 +2251,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="C18" s="10" t="n"/>
       <c r="D18" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -2482,21 +2267,13 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="G18" s="10" t="n"/>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>R, A</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -2534,11 +2311,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H19" s="10" t="n"/>
       <c r="I19" s="9" t="inlineStr">
         <is>
           <t>C</t>
@@ -2553,7 +2326,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -2571,26 +2344,10 @@
           <t>R</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2598,6 +2355,14 @@
           <t>Release</t>
         </is>
       </c>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -2729,17 +2494,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="H24" s="10" t="n"/>
       <c r="I24" s="10" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
@@ -2755,7 +2517,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Responsible — does the work to complete the task</t>
+          <t>Responsible - does the work to complete the task</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2529,7 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Accountable — owns the outcome, signs off, single owner per row</t>
+          <t>Accountable - owns the outcome and signs off; never more than one per row, exactly one on any row with a real decision or sign-off</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2541,7 @@
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Consulted — two-way input sought before/during the work</t>
+          <t>Consulted - two-way input sought before/during the work</t>
         </is>
       </c>
     </row>
@@ -2791,28 +2553,29 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Informed — kept updated on progress or outcome, one-way</t>
-        </is>
-      </c>
-    </row>
+          <t>Informed - kept updated on progress or outcome, one-way</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- Rules of thumb: exactly one A per row. R can be shared, A cannot.</t>
+          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>- If a role has no R/A/C/I on a row, leave the cell blank — do not mark every role on every row.</t>
+          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>- Validate row-by-row: no row with zero A, no row with more than one A.</t>
+          <t>- Validate row-by-row: no row with more than one A, and no row with a real decision or sign-off that has none.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2026-10-19: RACI workbook matches the templates
</commit_message>
<xml_diff>
--- a/RACI_Templates.xlsx
+++ b/RACI_Templates.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Copy this tab per project. Replace phase names/rows and roles as needed - keep one A per row.</t>
+          <t>Copy this tab per project. Replace phase names/rows and roles as needed - never more than one A per row.</t>
         </is>
       </c>
     </row>
@@ -837,12 +837,12 @@
       <c r="B10" s="10" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Accountable - owns the outcome, signs off, single owner per row</t>
+          <t>Accountable - owns the outcome and signs off; never more than one per row, exactly one on any row with a real decision or sign-off</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>- Rules of thumb: exactly one A per row. R can be shared, A cannot.</t>
+          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>- Validate row-by-row: no row with zero A, no row with more than one A.</t>
+          <t>- Validate row-by-row: no row with more than one A, and no row with a real decision or sign-off that has none.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2026-10-19: Consistency pass from the portfolio audit
Capacity cap: a large is a week elapsed with waits, the hands-on time leaves slack, and the illustrative baseline matches the cap (52 points). RACI: sponsor A only on business case, budget, baseline, go/no-go and closure (new go/no-go row); agile RACI gains a TPM column and a cross-team dependencies row; workbook updated to match. Kickoff: charter approval moves after the items it approves and is owned by the executive sponsor; phases approval is Must. RAID sample matches the guide's fields and the guide links it. Vendor guide: nineteen rows, Yellow not Amber. Same-repo absolute links made relative. Charter and kickoff "Where This Breaks" no longer repeat How to Fill It In.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C8u4r1uPPpTd4HU2JNuJEr
</commit_message>
<xml_diff>
--- a/RACI_Templates.xlsx
+++ b/RACI_Templates.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -884,7 +884,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A/R</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -1459,7 +1459,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Go-live execution</t>
+          <t>Go/no-go decision</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1482,9 +1482,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -1497,7 +1497,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1511,251 +1511,303 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t>Go-live execution</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t>Post-launch support/hypercare</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>A/R</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="n"/>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Closure</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="19" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Lessons learned</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I31" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J31" s="10" t="n"/>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
+          <t>Lessons learned</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>Project closure &amp; sign-off</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H32" s="10" t="n"/>
-      <c r="I32" s="10" t="n"/>
-      <c r="J32" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="n"/>
+      <c r="I33" s="10" t="n"/>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Responsible - does the work to complete the task</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Accountable - owns the outcome and signs off; never more than one per row, exactly one on any row with a real decision or sign-off</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Consulted - two-way input sought before/during the work</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Informed - kept updated on progress or outcome, one-way</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
-        <is>
-          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
-        </is>
-      </c>
-    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
+          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
+          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
           <t>- Validate row-by-row: no row with more than one A, and no row with a real decision or sign-off that has none.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A5:J5"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="B37:J37"/>
     <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A9:J9"/>
     <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A40:J40"/>
-    <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A26:J26"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A42:J42"/>
+    <mergeCell ref="A43:J43"/>
     <mergeCell ref="A41:J41"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="A13:J13"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="A42:J42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1767,7 +1819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1816,33 +1868,38 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
           <t>Dev Team</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>QA/Test</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Solution
 Architect</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Release
 Mgr</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Security/
 Compliance</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Stakeholders/
 Sponsor</t>
@@ -1862,7 +1919,8 @@
       <c r="F5" s="18" t="n"/>
       <c r="G5" s="18" t="n"/>
       <c r="H5" s="18" t="n"/>
-      <c r="I5" s="19" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1880,24 +1938,29 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1919,9 +1982,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -1945,6 +2008,11 @@
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1966,79 +2034,102 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="n"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="H8" s="10" t="n"/>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Cross-team dependencies &amp; risks</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>R, A</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Sprint Cadence</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="19" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Backlog refinement</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n"/>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Sprint planning</t>
+          <t>Backlog refinement</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -2048,17 +2139,13 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>R</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -2066,21 +2153,26 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="H11" s="10" t="n"/>
       <c r="I11" s="10" t="n"/>
+      <c r="J11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Daily standup</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n"/>
+          <t>Sprint planning</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
           <t>R</t>
@@ -2088,70 +2180,80 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="I12" s="10" t="n"/>
+      <c r="J12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Story/epic definition &amp; acceptance criteria</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Daily standup</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="10" t="n"/>
       <c r="I13" s="10" t="n"/>
+      <c r="J13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
+          <t>Story/epic definition &amp; acceptance criteria</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -2159,141 +2261,138 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G14" s="10" t="n"/>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n"/>
+      <c r="J14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Code review</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n"/>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n"/>
       <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Code review</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Quality &amp; Review</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
-      <c r="I16" s="19" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Sprint testing/QA</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>R, A</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Security scan/review</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
+          <t>Sprint testing/QA</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="C18" s="10" t="n"/>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="D18" s="10" t="n"/>
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>R, A</t>
         </is>
       </c>
       <c r="G18" s="10" t="n"/>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>R, A</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Sprint review/demo</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
+          <t>Security scan/review</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -2301,135 +2400,139 @@
           <t>C</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>R, A</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>Sprint review/demo</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
           <t>Sprint retrospective</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="10" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="10" t="n"/>
+      <c r="J21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="18" t="n"/>
-      <c r="I21" s="19" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Release readiness review</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Deployment/release</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Release readiness review</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -2442,17 +2545,22 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
         <is>
           <t>I</t>
         </is>
@@ -2461,139 +2569,196 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>Deployment/release</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>Post-release monitoring</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="I25" s="10" t="n"/>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Responsible - does the work to complete the task</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Accountable - owns the outcome and signs off; never more than one per row, exactly one on any row with a real decision or sign-off</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Consulted - two-way input sought before/during the work</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>Informed - kept updated on progress or outcome, one-way</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
-        </is>
-      </c>
-    </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
+          <t>- Rules of thumb: never more than one A per row. R can be shared, A cannot.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
+          <t>- If a role has no R/A/C/I on a row, leave the cell blank - do not mark every role on every row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
           <t>- Validate row-by-row: no row with more than one A, and no row with a real decision or sign-off that has none.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A34:I34"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>